<commit_message>
Add data for 2026-09-16
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -9,25 +9,25 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="South Shore" sheetId="3" r:id="rId3"/>
-    <sheet name="Albany Park" sheetId="4" r:id="rId4"/>
-    <sheet name="Old Town" sheetId="5" r:id="rId5"/>
-    <sheet name="Loop" sheetId="6" r:id="rId6"/>
-    <sheet name="O'Hare" sheetId="7" r:id="rId7"/>
-    <sheet name="Near South Side" sheetId="8" r:id="rId8"/>
-    <sheet name="Grand Crossing" sheetId="9" r:id="rId9"/>
-    <sheet name="Austin" sheetId="10" r:id="rId10"/>
-    <sheet name="Avondale" sheetId="11" r:id="rId11"/>
-    <sheet name="Rush &amp; Division" sheetId="12" r:id="rId12"/>
-    <sheet name="Oakland" sheetId="13" r:id="rId13"/>
-    <sheet name="Chatham" sheetId="14" r:id="rId14"/>
-    <sheet name="New City" sheetId="15" r:id="rId15"/>
-    <sheet name="Belmont Cragin" sheetId="16" r:id="rId16"/>
-    <sheet name="Woodlawn" sheetId="17" r:id="rId17"/>
-    <sheet name="West Loop" sheetId="18" r:id="rId18"/>
-    <sheet name="Uptown" sheetId="19" r:id="rId19"/>
-    <sheet name="Lake View" sheetId="20" r:id="rId20"/>
-    <sheet name="North Lawndale" sheetId="21" r:id="rId21"/>
+    <sheet name="Albany Park" sheetId="3" r:id="rId3"/>
+    <sheet name="Woodlawn" sheetId="4" r:id="rId4"/>
+    <sheet name="North Lawndale" sheetId="5" r:id="rId5"/>
+    <sheet name="South Shore" sheetId="6" r:id="rId6"/>
+    <sheet name="Old Town" sheetId="7" r:id="rId7"/>
+    <sheet name="Loop" sheetId="8" r:id="rId8"/>
+    <sheet name="O'Hare" sheetId="9" r:id="rId9"/>
+    <sheet name="Near South Side" sheetId="10" r:id="rId10"/>
+    <sheet name="Grand Crossing" sheetId="11" r:id="rId11"/>
+    <sheet name="Austin" sheetId="12" r:id="rId12"/>
+    <sheet name="Avondale" sheetId="13" r:id="rId13"/>
+    <sheet name="Rush &amp; Division" sheetId="14" r:id="rId14"/>
+    <sheet name="Oakland" sheetId="15" r:id="rId15"/>
+    <sheet name="Chatham" sheetId="16" r:id="rId16"/>
+    <sheet name="New City" sheetId="17" r:id="rId17"/>
+    <sheet name="Belmont Cragin" sheetId="18" r:id="rId18"/>
+    <sheet name="West Loop" sheetId="19" r:id="rId19"/>
+    <sheet name="Uptown" sheetId="20" r:id="rId20"/>
+    <sheet name="Lake View" sheetId="21" r:id="rId21"/>
     <sheet name="Grand Boulevard" sheetId="22" r:id="rId22"/>
     <sheet name="West Town" sheetId="23" r:id="rId23"/>
     <sheet name="Englewood" sheetId="24" r:id="rId24"/>
@@ -889,7 +889,7 @@
         <v>137</v>
       </c>
       <c r="M2">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1050,7 +1050,7 @@
         <v>467</v>
       </c>
       <c r="M6">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>896</v>
       </c>
       <c r="M7">
-        <v>454</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -1164,41 +1164,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
       <c r="F2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>7</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1206,62 +1191,41 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>7</v>
-      </c>
-      <c r="F3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>12</v>
-      </c>
-      <c r="L3">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
       <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="M4">
         <v>1</v>
       </c>
     </row>
@@ -1278,40 +1242,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1319,40 +1283,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="E7">
-        <v>57</v>
+        <v>7</v>
       </c>
       <c r="F7">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="G7">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="H7">
-        <v>63</v>
+        <v>9</v>
       </c>
       <c r="I7">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="J7">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="K7">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="L7">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="M7">
-        <v>36</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1361,6 +1325,534 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>7</v>
+      </c>
+      <c r="K2">
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3">
+        <v>19</v>
+      </c>
+      <c r="G3">
+        <v>9</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>17</v>
+      </c>
+      <c r="L3">
+        <v>13</v>
+      </c>
+      <c r="M3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>37</v>
+      </c>
+      <c r="D6">
+        <v>21</v>
+      </c>
+      <c r="E6">
+        <v>22</v>
+      </c>
+      <c r="F6">
+        <v>27</v>
+      </c>
+      <c r="G6">
+        <v>15</v>
+      </c>
+      <c r="H6">
+        <v>25</v>
+      </c>
+      <c r="I6">
+        <v>21</v>
+      </c>
+      <c r="J6">
+        <v>26</v>
+      </c>
+      <c r="K6">
+        <v>49</v>
+      </c>
+      <c r="L6">
+        <v>44</v>
+      </c>
+      <c r="M6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>42</v>
+      </c>
+      <c r="D7">
+        <v>36</v>
+      </c>
+      <c r="E7">
+        <v>38</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>28</v>
+      </c>
+      <c r="H7">
+        <v>39</v>
+      </c>
+      <c r="I7">
+        <v>39</v>
+      </c>
+      <c r="J7">
+        <v>47</v>
+      </c>
+      <c r="K7">
+        <v>74</v>
+      </c>
+      <c r="L7">
+        <v>63</v>
+      </c>
+      <c r="M7">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>8</v>
+      </c>
+      <c r="K2">
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
+      <c r="M2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
+        <v>14</v>
+      </c>
+      <c r="M3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>31</v>
+      </c>
+      <c r="D6">
+        <v>22</v>
+      </c>
+      <c r="E6">
+        <v>44</v>
+      </c>
+      <c r="F6">
+        <v>38</v>
+      </c>
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6">
+        <v>50</v>
+      </c>
+      <c r="I6">
+        <v>34</v>
+      </c>
+      <c r="J6">
+        <v>26</v>
+      </c>
+      <c r="K6">
+        <v>24</v>
+      </c>
+      <c r="L6">
+        <v>14</v>
+      </c>
+      <c r="M6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>40</v>
+      </c>
+      <c r="D7">
+        <v>32</v>
+      </c>
+      <c r="E7">
+        <v>57</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>34</v>
+      </c>
+      <c r="H7">
+        <v>63</v>
+      </c>
+      <c r="I7">
+        <v>44</v>
+      </c>
+      <c r="J7">
+        <v>47</v>
+      </c>
+      <c r="K7">
+        <v>46</v>
+      </c>
+      <c r="L7">
+        <v>33</v>
+      </c>
+      <c r="M7">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1571,7 +2063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1788,7 +2280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1882,7 +2374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2134,7 +2626,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2318,7 +2810,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2476,224 +2968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
-      <c r="I3">
-        <v>5</v>
-      </c>
-      <c r="J3">
-        <v>5</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>11</v>
-      </c>
-      <c r="C5">
-        <v>12</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>9</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>6</v>
-      </c>
-      <c r="K5">
-        <v>7</v>
-      </c>
-      <c r="L5">
-        <v>4</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>16</v>
-      </c>
-      <c r="C6">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>11</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>11</v>
-      </c>
-      <c r="J6">
-        <v>11</v>
-      </c>
-      <c r="K6">
-        <v>12</v>
-      </c>
-      <c r="L6">
-        <v>5</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2923,241 +3198,6 @@
       </c>
       <c r="M7">
         <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>4</v>
-      </c>
-      <c r="K2">
-        <v>5</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-      <c r="G3">
-        <v>6</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>7</v>
-      </c>
-      <c r="K3">
-        <v>7</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>9</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5">
-        <v>6</v>
-      </c>
-      <c r="G5">
-        <v>14</v>
-      </c>
-      <c r="H5">
-        <v>7</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>11</v>
-      </c>
-      <c r="L5">
-        <v>8</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>14</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6">
-        <v>11</v>
-      </c>
-      <c r="F6">
-        <v>10</v>
-      </c>
-      <c r="G6">
-        <v>22</v>
-      </c>
-      <c r="H6">
-        <v>14</v>
-      </c>
-      <c r="I6">
-        <v>10</v>
-      </c>
-      <c r="J6">
-        <v>16</v>
-      </c>
-      <c r="K6">
-        <v>23</v>
-      </c>
-      <c r="L6">
-        <v>13</v>
-      </c>
-      <c r="M6">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -3261,7 +3301,7 @@
         <v>3</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -5337,7 +5377,7 @@
         <v>18</v>
       </c>
       <c r="M65">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -6440,7 +6480,7 @@
         <v>5</v>
       </c>
       <c r="M96">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -6522,7 +6562,7 @@
         <v>896</v>
       </c>
       <c r="M98">
-        <v>454</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -6694,6 +6734,9 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
       <c r="C2">
         <v>4</v>
       </c>
@@ -6701,133 +6744,118 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
       <c r="C3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
         <v>7</v>
       </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>11</v>
-      </c>
       <c r="K3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
+      <c r="B4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
       <c r="C5">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>6</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="G5">
         <v>14</v>
       </c>
-      <c r="D5">
-        <v>12</v>
-      </c>
-      <c r="E5">
-        <v>10</v>
-      </c>
-      <c r="F5">
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
         <v>11</v>
       </c>
-      <c r="G5">
-        <v>11</v>
-      </c>
-      <c r="H5">
-        <v>17</v>
-      </c>
-      <c r="I5">
-        <v>20</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>10</v>
-      </c>
       <c r="L5">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -6835,40 +6863,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C6">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="G6">
+        <v>22</v>
+      </c>
+      <c r="H6">
         <v>14</v>
       </c>
-      <c r="E6">
-        <v>18</v>
-      </c>
-      <c r="F6">
-        <v>18</v>
-      </c>
-      <c r="G6">
-        <v>19</v>
-      </c>
-      <c r="H6">
-        <v>27</v>
-      </c>
       <c r="I6">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="J6">
         <v>16</v>
       </c>
       <c r="K6">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L6">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="M6">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -6941,41 +6969,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6983,89 +7008,101 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L3">
         <v>7</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
       <c r="H4">
         <v>1</v>
       </c>
-      <c r="J4">
-        <v>1</v>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
+      <c r="C5">
+        <v>14</v>
+      </c>
+      <c r="D5">
         <v>12</v>
       </c>
-      <c r="C5">
-        <v>21</v>
-      </c>
-      <c r="D5">
-        <v>28</v>
-      </c>
       <c r="E5">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F5">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="G5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H5">
+        <v>17</v>
+      </c>
+      <c r="I5">
+        <v>20</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="K5">
         <v>10</v>
       </c>
-      <c r="I5">
-        <v>15</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>9</v>
-      </c>
       <c r="L5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -7073,40 +7110,40 @@
         <v>6</v>
       </c>
       <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>23</v>
+      </c>
+      <c r="D6">
         <v>14</v>
       </c>
-      <c r="C6">
+      <c r="E6">
+        <v>18</v>
+      </c>
+      <c r="F6">
+        <v>18</v>
+      </c>
+      <c r="G6">
+        <v>19</v>
+      </c>
+      <c r="H6">
+        <v>27</v>
+      </c>
+      <c r="I6">
         <v>26</v>
       </c>
-      <c r="D6">
-        <v>29</v>
-      </c>
-      <c r="E6">
+      <c r="J6">
+        <v>16</v>
+      </c>
+      <c r="K6">
         <v>24</v>
       </c>
-      <c r="F6">
-        <v>42</v>
-      </c>
-      <c r="G6">
-        <v>18</v>
-      </c>
-      <c r="H6">
-        <v>18</v>
-      </c>
-      <c r="I6">
-        <v>21</v>
-      </c>
-      <c r="J6">
+      <c r="L6">
+        <v>20</v>
+      </c>
+      <c r="M6">
         <v>12</v>
-      </c>
-      <c r="K6">
-        <v>18</v>
-      </c>
-      <c r="L6">
-        <v>18</v>
-      </c>
-      <c r="M6">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -8921,10 +8958,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -8936,10 +8973,9 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8962,42 +8998,30 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="I1" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="J1" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="K1" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -9006,142 +9030,126 @@
         <v>2</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2">
         <v>2</v>
       </c>
-      <c r="M2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>3</v>
-      </c>
-      <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>6</v>
-      </c>
-      <c r="M3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>11</v>
-      </c>
-      <c r="C4">
-        <v>10</v>
-      </c>
-      <c r="D4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
+        <v>9</v>
+      </c>
+      <c r="J6">
         <v>7</v>
       </c>
-      <c r="F4">
-        <v>7</v>
-      </c>
-      <c r="G4">
-        <v>7</v>
-      </c>
-      <c r="H4">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>8</v>
-      </c>
-      <c r="J4">
-        <v>12</v>
-      </c>
-      <c r="K4">
-        <v>4</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>15</v>
-      </c>
-      <c r="C5">
-        <v>15</v>
-      </c>
-      <c r="D5">
-        <v>12</v>
-      </c>
-      <c r="E5">
-        <v>11</v>
-      </c>
-      <c r="F5">
-        <v>12</v>
-      </c>
-      <c r="G5">
-        <v>9</v>
-      </c>
-      <c r="H5">
-        <v>11</v>
-      </c>
-      <c r="I5">
-        <v>12</v>
-      </c>
-      <c r="J5">
-        <v>15</v>
-      </c>
-      <c r="K5">
-        <v>9</v>
-      </c>
-      <c r="L5">
-        <v>9</v>
-      </c>
-      <c r="M5">
-        <v>8</v>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -11427,7 +11435,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -11442,9 +11450,10 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -11467,157 +11476,172 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2">
-        <v>1</v>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
         <v>2</v>
       </c>
       <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
         <v>2</v>
       </c>
       <c r="L2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>2</v>
+      </c>
       <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
       </c>
       <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>5</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>7</v>
       </c>
       <c r="L5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I6">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J6">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
         <v>4</v>
       </c>
     </row>
@@ -13581,25 +13605,40 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L2">
+        <v>4</v>
+      </c>
+      <c r="M2">
         <v>2</v>
       </c>
     </row>
@@ -13610,31 +13649,34 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>3</v>
+      <c r="C3">
+        <v>2</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L3">
+        <v>7</v>
+      </c>
+      <c r="M3">
         <v>3</v>
       </c>
     </row>
@@ -13642,6 +13684,9 @@
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
       <c r="J4">
         <v>1</v>
       </c>
@@ -13651,40 +13696,40 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="C5">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="E5">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F5">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="G5">
         <v>12</v>
       </c>
       <c r="H5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I5">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M5">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13692,40 +13737,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D6">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E6">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F6">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="G6">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H6">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I6">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J6">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K6">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="L6">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -15200,10 +15245,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -15264,40 +15309,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="L2">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15305,177 +15350,122 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="L3">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>11</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="G4">
+        <v>7</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>15</v>
+      </c>
+      <c r="C5">
+        <v>15</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
+      </c>
+      <c r="E5">
+        <v>11</v>
+      </c>
+      <c r="F5">
+        <v>12</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>11</v>
+      </c>
+      <c r="I5">
+        <v>12</v>
       </c>
       <c r="J5">
-        <v>2</v>
+        <v>15</v>
+      </c>
+      <c r="K5">
+        <v>9</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>30</v>
-      </c>
-      <c r="C6">
-        <v>44</v>
-      </c>
-      <c r="D6">
-        <v>49</v>
-      </c>
-      <c r="E6">
-        <v>67</v>
-      </c>
-      <c r="F6">
-        <v>69</v>
-      </c>
-      <c r="G6">
-        <v>57</v>
-      </c>
-      <c r="H6">
-        <v>80</v>
-      </c>
-      <c r="I6">
-        <v>80</v>
-      </c>
-      <c r="J6">
-        <v>64</v>
-      </c>
-      <c r="K6">
-        <v>48</v>
-      </c>
-      <c r="L6">
-        <v>44</v>
-      </c>
-      <c r="M6">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>49</v>
-      </c>
-      <c r="C7">
-        <v>62</v>
-      </c>
-      <c r="D7">
-        <v>79</v>
-      </c>
-      <c r="E7">
-        <v>92</v>
-      </c>
-      <c r="F7">
-        <v>92</v>
-      </c>
-      <c r="G7">
-        <v>88</v>
-      </c>
-      <c r="H7">
-        <v>120</v>
-      </c>
-      <c r="I7">
-        <v>130</v>
-      </c>
-      <c r="J7">
-        <v>131</v>
-      </c>
-      <c r="K7">
-        <v>91</v>
-      </c>
-      <c r="L7">
-        <v>100</v>
-      </c>
-      <c r="M7">
-        <v>45</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -17227,7 +17217,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -17242,9 +17232,10 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -17264,163 +17255,176 @@
         <v>2019</v>
       </c>
       <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
         <v>2021</v>
       </c>
-      <c r="H1" s="1">
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="D2">
         <v>2</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
       <c r="H2">
-        <v>3</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L2">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3">
-        <v>1</v>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
       <c r="J4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>17</v>
+      </c>
+      <c r="F5">
+        <v>18</v>
+      </c>
+      <c r="G5">
+        <v>12</v>
+      </c>
+      <c r="H5">
+        <v>12</v>
+      </c>
+      <c r="I5">
+        <v>17</v>
+      </c>
+      <c r="J5">
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>17</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6">
+        <v>19</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>17</v>
+      </c>
+      <c r="I6">
+        <v>19</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>14</v>
+      </c>
+      <c r="K6">
+        <v>24</v>
       </c>
       <c r="L6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
-        <v>6</v>
-      </c>
-      <c r="G7">
-        <v>3</v>
-      </c>
-      <c r="H7">
-        <v>7</v>
-      </c>
-      <c r="I7">
-        <v>3</v>
-      </c>
-      <c r="J7">
-        <v>5</v>
-      </c>
-      <c r="K7">
-        <v>9</v>
-      </c>
-      <c r="L7">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -19081,23 +19085,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
       <c r="F2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>15</v>
+      </c>
+      <c r="L2">
+        <v>15</v>
       </c>
       <c r="M2">
         <v>2</v>
@@ -19108,49 +19127,94 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>26</v>
+      </c>
+      <c r="L3">
+        <v>34</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>5</v>
+      </c>
+      <c r="M4">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K5">
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -19159,40 +19223,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>67</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="I6">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -19200,40 +19264,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>7</v>
+        <v>49</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="D7">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="E7">
-        <v>7</v>
+        <v>92</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>92</v>
       </c>
       <c r="G7">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="H7">
-        <v>9</v>
+        <v>120</v>
       </c>
       <c r="I7">
-        <v>13</v>
+        <v>130</v>
       </c>
       <c r="J7">
-        <v>8</v>
+        <v>131</v>
       </c>
       <c r="K7">
-        <v>8</v>
+        <v>91</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="M7">
-        <v>7</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -20322,7 +20386,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -20337,10 +20401,9 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -20360,226 +20423,163 @@
         <v>2019</v>
       </c>
       <c r="G1" s="1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="H1" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="I1" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="J1" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="K1" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
         <v>7</v>
       </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>6</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>7</v>
-      </c>
-      <c r="K2">
-        <v>7</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>8</v>
-      </c>
-      <c r="E3">
+      <c r="I7">
+        <v>3</v>
+      </c>
+      <c r="J7">
+        <v>5</v>
+      </c>
+      <c r="K7">
         <v>9</v>
       </c>
-      <c r="F3">
-        <v>19</v>
-      </c>
-      <c r="G3">
+      <c r="L7">
         <v>9</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>13</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>17</v>
-      </c>
-      <c r="L3">
-        <v>13</v>
-      </c>
-      <c r="M3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>24</v>
-      </c>
-      <c r="C6">
-        <v>37</v>
-      </c>
-      <c r="D6">
-        <v>21</v>
-      </c>
-      <c r="E6">
-        <v>22</v>
-      </c>
-      <c r="F6">
-        <v>27</v>
-      </c>
-      <c r="G6">
-        <v>15</v>
-      </c>
-      <c r="H6">
-        <v>25</v>
-      </c>
-      <c r="I6">
-        <v>21</v>
-      </c>
-      <c r="J6">
-        <v>26</v>
-      </c>
-      <c r="K6">
-        <v>49</v>
-      </c>
-      <c r="L6">
-        <v>44</v>
-      </c>
-      <c r="M6">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
-        <v>42</v>
-      </c>
-      <c r="D7">
-        <v>36</v>
-      </c>
-      <c r="E7">
-        <v>38</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>28</v>
-      </c>
-      <c r="H7">
-        <v>39</v>
-      </c>
-      <c r="I7">
-        <v>39</v>
-      </c>
-      <c r="J7">
-        <v>47</v>
-      </c>
-      <c r="K7">
-        <v>74</v>
-      </c>
-      <c r="L7">
-        <v>63</v>
-      </c>
-      <c r="M7">
-        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-19
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -9,27 +9,27 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Austin" sheetId="3" r:id="rId3"/>
-    <sheet name="Roseland" sheetId="4" r:id="rId4"/>
-    <sheet name="Albany Park" sheetId="5" r:id="rId5"/>
-    <sheet name="Woodlawn" sheetId="6" r:id="rId6"/>
-    <sheet name="North Lawndale" sheetId="7" r:id="rId7"/>
-    <sheet name="South Shore" sheetId="8" r:id="rId8"/>
-    <sheet name="Old Town" sheetId="9" r:id="rId9"/>
-    <sheet name="Loop" sheetId="10" r:id="rId10"/>
-    <sheet name="O'Hare" sheetId="11" r:id="rId11"/>
-    <sheet name="Near South Side" sheetId="12" r:id="rId12"/>
-    <sheet name="Grand Crossing" sheetId="13" r:id="rId13"/>
-    <sheet name="Avondale" sheetId="14" r:id="rId14"/>
-    <sheet name="Rush &amp; Division" sheetId="15" r:id="rId15"/>
-    <sheet name="Oakland" sheetId="16" r:id="rId16"/>
-    <sheet name="Chatham" sheetId="17" r:id="rId17"/>
-    <sheet name="New City" sheetId="18" r:id="rId18"/>
-    <sheet name="Belmont Cragin" sheetId="19" r:id="rId19"/>
-    <sheet name="West Loop" sheetId="20" r:id="rId20"/>
-    <sheet name="Uptown" sheetId="21" r:id="rId21"/>
-    <sheet name="Hegewisch" sheetId="22" r:id="rId22"/>
-    <sheet name="Lake View" sheetId="23" r:id="rId23"/>
+    <sheet name="Lake View" sheetId="3" r:id="rId3"/>
+    <sheet name="Austin" sheetId="4" r:id="rId4"/>
+    <sheet name="Roseland" sheetId="5" r:id="rId5"/>
+    <sheet name="Albany Park" sheetId="6" r:id="rId6"/>
+    <sheet name="Woodlawn" sheetId="7" r:id="rId7"/>
+    <sheet name="North Lawndale" sheetId="8" r:id="rId8"/>
+    <sheet name="South Shore" sheetId="9" r:id="rId9"/>
+    <sheet name="Old Town" sheetId="10" r:id="rId10"/>
+    <sheet name="Loop" sheetId="11" r:id="rId11"/>
+    <sheet name="O'Hare" sheetId="12" r:id="rId12"/>
+    <sheet name="Near South Side" sheetId="13" r:id="rId13"/>
+    <sheet name="Grand Crossing" sheetId="14" r:id="rId14"/>
+    <sheet name="Avondale" sheetId="15" r:id="rId15"/>
+    <sheet name="Rush &amp; Division" sheetId="16" r:id="rId16"/>
+    <sheet name="Oakland" sheetId="17" r:id="rId17"/>
+    <sheet name="Chatham" sheetId="18" r:id="rId18"/>
+    <sheet name="New City" sheetId="19" r:id="rId19"/>
+    <sheet name="Belmont Cragin" sheetId="20" r:id="rId20"/>
+    <sheet name="West Loop" sheetId="21" r:id="rId21"/>
+    <sheet name="Uptown" sheetId="22" r:id="rId22"/>
+    <sheet name="Hegewisch" sheetId="23" r:id="rId23"/>
     <sheet name="Grand Boulevard" sheetId="24" r:id="rId24"/>
     <sheet name="West Town" sheetId="25" r:id="rId25"/>
     <sheet name="Englewood" sheetId="26" r:id="rId26"/>
@@ -1050,7 +1050,7 @@
         <v>467</v>
       </c>
       <c r="M6">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>896</v>
       </c>
       <c r="M7">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -1100,6 +1100,223 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>4</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>6</v>
+      </c>
+      <c r="K3">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>17</v>
+      </c>
+      <c r="F5">
+        <v>18</v>
+      </c>
+      <c r="G5">
+        <v>12</v>
+      </c>
+      <c r="H5">
+        <v>12</v>
+      </c>
+      <c r="I5">
+        <v>17</v>
+      </c>
+      <c r="J5">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>17</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>9</v>
+      </c>
+      <c r="E6">
+        <v>19</v>
+      </c>
+      <c r="F6">
+        <v>24</v>
+      </c>
+      <c r="G6">
+        <v>15</v>
+      </c>
+      <c r="H6">
+        <v>17</v>
+      </c>
+      <c r="I6">
+        <v>19</v>
+      </c>
+      <c r="J6">
+        <v>14</v>
+      </c>
+      <c r="K6">
+        <v>24</v>
+      </c>
+      <c r="L6">
+        <v>10</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1384,7 +1601,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1580,231 +1797,6 @@
       </c>
       <c r="L7">
         <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>6</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>6</v>
-      </c>
-      <c r="I6">
-        <v>8</v>
-      </c>
-      <c r="J6">
-        <v>4</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>7</v>
-      </c>
-      <c r="C7">
-        <v>3</v>
-      </c>
-      <c r="D7">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>7</v>
-      </c>
-      <c r="F7">
-        <v>5</v>
-      </c>
-      <c r="G7">
-        <v>8</v>
-      </c>
-      <c r="H7">
-        <v>9</v>
-      </c>
-      <c r="I7">
-        <v>13</v>
-      </c>
-      <c r="J7">
-        <v>8</v>
-      </c>
-      <c r="K7">
-        <v>8</v>
-      </c>
-      <c r="L7">
-        <v>4</v>
-      </c>
-      <c r="M7">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1877,41 +1869,26 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2">
-        <v>7</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
       <c r="F2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>7</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1919,56 +1896,41 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>9</v>
-      </c>
-      <c r="F3">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>17</v>
-      </c>
-      <c r="L3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
       <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="M4">
         <v>1</v>
       </c>
     </row>
@@ -1976,19 +1938,7 @@
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
       <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -1997,40 +1947,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>27</v>
+        <v>4</v>
       </c>
       <c r="G6">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="J6">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="L6">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2038,40 +1988,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E7">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="F7">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="G7">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="H7">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="I7">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="J7">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="K7">
-        <v>74</v>
+        <v>8</v>
       </c>
       <c r="L7">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="M7">
-        <v>27</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2081,7 +2031,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -2145,144 +2095,200 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
       <c r="E3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>17</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>5</v>
-      </c>
       <c r="I5">
-        <v>3</v>
-      </c>
-      <c r="J5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="J6">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>42</v>
+      </c>
+      <c r="D7">
+        <v>36</v>
+      </c>
+      <c r="E7">
+        <v>38</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>28</v>
+      </c>
+      <c r="H7">
+        <v>39</v>
+      </c>
+      <c r="I7">
+        <v>39</v>
+      </c>
+      <c r="J7">
+        <v>47</v>
+      </c>
+      <c r="K7">
+        <v>74</v>
+      </c>
+      <c r="L7">
+        <v>63</v>
+      </c>
+      <c r="M7">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2356,67 +2362,64 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>2</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>2</v>
       </c>
       <c r="L3">
         <v>2</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="M4">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="K4">
         <v>1</v>
       </c>
     </row>
@@ -2425,40 +2428,37 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D5">
         <v>3</v>
       </c>
       <c r="E5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K5">
         <v>3</v>
       </c>
       <c r="L5">
-        <v>5</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2466,40 +2466,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G6">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="J6">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2508,6 +2508,223 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>7</v>
+      </c>
+      <c r="F5">
+        <v>9</v>
+      </c>
+      <c r="G5">
+        <v>14</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
+      </c>
+      <c r="I5">
+        <v>9</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>13</v>
+      </c>
+      <c r="G6">
+        <v>16</v>
+      </c>
+      <c r="H6">
+        <v>11</v>
+      </c>
+      <c r="I6">
+        <v>14</v>
+      </c>
+      <c r="J6">
+        <v>6</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>7</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2601,7 +2818,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2853,7 +3070,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3030,164 +3247,6 @@
       </c>
       <c r="L5">
         <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>6</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6">
-        <v>7</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6">
-        <v>3</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
-        <v>6</v>
-      </c>
-      <c r="I6">
-        <v>2</v>
-      </c>
-      <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4740,7 +4799,7 @@
         <v>20</v>
       </c>
       <c r="M47">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -6555,7 +6614,7 @@
         <v>896</v>
       </c>
       <c r="M98">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
   </sheetData>
@@ -6664,6 +6723,164 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>6</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>7</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -6899,7 +7116,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7134,7 +7351,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7205,253 +7422,6 @@
       </c>
       <c r="E5">
         <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>3</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>6</v>
-      </c>
-      <c r="L2">
-        <v>6</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>5</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>11</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>14</v>
-      </c>
-      <c r="D5">
-        <v>12</v>
-      </c>
-      <c r="E5">
-        <v>10</v>
-      </c>
-      <c r="F5">
-        <v>11</v>
-      </c>
-      <c r="G5">
-        <v>11</v>
-      </c>
-      <c r="H5">
-        <v>17</v>
-      </c>
-      <c r="I5">
-        <v>20</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>10</v>
-      </c>
-      <c r="L5">
-        <v>5</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>23</v>
-      </c>
-      <c r="D6">
-        <v>14</v>
-      </c>
-      <c r="E6">
-        <v>18</v>
-      </c>
-      <c r="F6">
-        <v>18</v>
-      </c>
-      <c r="G6">
-        <v>19</v>
-      </c>
-      <c r="H6">
-        <v>27</v>
-      </c>
-      <c r="I6">
-        <v>26</v>
-      </c>
-      <c r="J6">
-        <v>16</v>
-      </c>
-      <c r="K6">
-        <v>24</v>
-      </c>
-      <c r="L6">
-        <v>20</v>
-      </c>
-      <c r="M6">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -8806,7 +8776,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -8869,41 +8839,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>4</v>
-      </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -8911,59 +8878,59 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
         <v>7</v>
       </c>
-      <c r="F3">
-        <v>6</v>
-      </c>
-      <c r="G3">
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>11</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
         <v>7</v>
       </c>
-      <c r="H3">
-        <v>8</v>
-      </c>
-      <c r="I3">
-        <v>6</v>
-      </c>
-      <c r="J3">
-        <v>10</v>
-      </c>
-      <c r="K3">
-        <v>12</v>
-      </c>
-      <c r="L3">
-        <v>14</v>
-      </c>
       <c r="M3">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
       </c>
       <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
         <v>2</v>
       </c>
       <c r="M4">
@@ -8972,92 +8939,81 @@
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>11</v>
+      </c>
+      <c r="H5">
+        <v>17</v>
+      </c>
+      <c r="I5">
+        <v>20</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="L5">
+        <v>5</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
         <v>23</v>
       </c>
-      <c r="C6">
-        <v>31</v>
-      </c>
       <c r="D6">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E6">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="F6">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="G6">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="H6">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="I6">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="J6">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="K6">
         <v>24</v>
       </c>
       <c r="L6">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="M6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
-        <v>40</v>
-      </c>
-      <c r="D7">
-        <v>32</v>
-      </c>
-      <c r="E7">
-        <v>57</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>34</v>
-      </c>
-      <c r="H7">
-        <v>63</v>
-      </c>
-      <c r="I7">
-        <v>44</v>
-      </c>
-      <c r="J7">
-        <v>47</v>
-      </c>
-      <c r="K7">
-        <v>46</v>
-      </c>
-      <c r="L7">
-        <v>33</v>
-      </c>
-      <c r="M7">
-        <v>37</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -11386,40 +11342,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>8</v>
+      </c>
+      <c r="K2">
         <v>7</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
       <c r="L2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -11427,73 +11383,70 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F3">
+        <v>6</v>
+      </c>
+      <c r="G3">
         <v>7</v>
       </c>
-      <c r="G3">
-        <v>6</v>
-      </c>
       <c r="H3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
         <v>14</v>
       </c>
-      <c r="K3">
-        <v>7</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
-      </c>
       <c r="M3">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>2</v>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="K5">
         <v>1</v>
       </c>
     </row>
@@ -11502,40 +11455,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C6">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="D6">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E6">
+        <v>44</v>
+      </c>
+      <c r="F6">
+        <v>38</v>
+      </c>
+      <c r="G6">
+        <v>24</v>
+      </c>
+      <c r="H6">
+        <v>50</v>
+      </c>
+      <c r="I6">
+        <v>34</v>
+      </c>
+      <c r="J6">
+        <v>26</v>
+      </c>
+      <c r="K6">
+        <v>24</v>
+      </c>
+      <c r="L6">
         <v>14</v>
       </c>
-      <c r="F6">
-        <v>12</v>
-      </c>
-      <c r="G6">
-        <v>14</v>
-      </c>
-      <c r="H6">
-        <v>19</v>
-      </c>
-      <c r="I6">
-        <v>29</v>
-      </c>
-      <c r="J6">
-        <v>19</v>
-      </c>
-      <c r="K6">
-        <v>20</v>
-      </c>
-      <c r="L6">
-        <v>26</v>
-      </c>
       <c r="M6">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -11543,40 +11496,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D7">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="F7">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="G7">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="H7">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="I7">
+        <v>44</v>
+      </c>
+      <c r="J7">
         <v>47</v>
       </c>
-      <c r="J7">
-        <v>35</v>
-      </c>
       <c r="K7">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="L7">
+        <v>33</v>
+      </c>
+      <c r="M7">
         <v>37</v>
-      </c>
-      <c r="M7">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -13473,7 +13426,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -13488,9 +13441,10 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -13513,158 +13467,220 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>3</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>7</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="J3">
+        <v>14</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>7</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4">
-        <v>2</v>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>3</v>
-      </c>
-      <c r="J5">
-        <v>4</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="I6">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="J6">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>26</v>
+      </c>
+      <c r="M6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>26</v>
+      </c>
+      <c r="C7">
+        <v>25</v>
+      </c>
+      <c r="D7">
+        <v>16</v>
+      </c>
+      <c r="E7">
+        <v>23</v>
+      </c>
+      <c r="F7">
+        <v>23</v>
+      </c>
+      <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <v>31</v>
+      </c>
+      <c r="I7">
+        <v>47</v>
+      </c>
+      <c r="J7">
+        <v>35</v>
+      </c>
+      <c r="K7">
+        <v>31</v>
+      </c>
+      <c r="L7">
+        <v>37</v>
+      </c>
+      <c r="M7">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -15179,7 +15195,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -15194,10 +15210,9 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -15220,173 +15235,158 @@
         <v>2020</v>
       </c>
       <c r="H1" s="1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="I1" s="1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="J1" s="1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="K1" s="1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
+      <c r="D2">
+        <v>1</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>2</v>
       </c>
       <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
         <v>2</v>
       </c>
       <c r="L2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="F3">
-        <v>2</v>
-      </c>
       <c r="G3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>5</v>
-      </c>
-      <c r="J3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="M3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6">
         <v>9</v>
       </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>4</v>
-      </c>
-      <c r="J5">
-        <v>6</v>
-      </c>
-      <c r="K5">
+      <c r="J6">
         <v>7</v>
       </c>
-      <c r="L5">
-        <v>4</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>16</v>
-      </c>
-      <c r="C6">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>11</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>8</v>
-      </c>
-      <c r="I6">
-        <v>11</v>
-      </c>
-      <c r="J6">
-        <v>11</v>
-      </c>
       <c r="K6">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L6">
         <v>5</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -17278,40 +17278,22 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>3</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
-      </c>
-      <c r="H2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I2">
         <v>2</v>
       </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
       <c r="L2">
-        <v>4</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -17319,47 +17301,44 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G3">
         <v>3</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J3">
         <v>5</v>
       </c>
       <c r="K3">
-        <v>6</v>
-      </c>
-      <c r="L3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
       <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="J4">
         <v>1</v>
       </c>
     </row>
@@ -17368,40 +17347,40 @@
         <v>5</v>
       </c>
       <c r="B5">
+        <v>11</v>
+      </c>
+      <c r="C5">
         <v>12</v>
       </c>
-      <c r="C5">
-        <v>21</v>
-      </c>
       <c r="D5">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="E5">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="F5">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I5">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L5">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -17409,40 +17388,40 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E6">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F6">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="G6">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="J6">
+        <v>11</v>
+      </c>
+      <c r="K6">
         <v>12</v>
       </c>
-      <c r="K6">
-        <v>18</v>
-      </c>
       <c r="L6">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -18991,10 +18970,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -19055,10 +19034,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -19070,10 +19049,10 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I2">
         <v>2</v>
@@ -19082,13 +19061,13 @@
         <v>1</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -19096,37 +19075,34 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M3">
         <v>3</v>
@@ -19134,83 +19110,94 @@
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>11</v>
-      </c>
-      <c r="C4">
-        <v>10</v>
-      </c>
-      <c r="D4">
-        <v>6</v>
-      </c>
-      <c r="E4">
-        <v>7</v>
-      </c>
-      <c r="F4">
-        <v>7</v>
-      </c>
-      <c r="G4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H4">
-        <v>3</v>
-      </c>
-      <c r="I4">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J4">
-        <v>12</v>
-      </c>
-      <c r="K4">
-        <v>4</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>21</v>
+      </c>
+      <c r="D5">
+        <v>28</v>
+      </c>
+      <c r="E5">
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>35</v>
+      </c>
+      <c r="G5">
+        <v>12</v>
+      </c>
+      <c r="H5">
+        <v>10</v>
+      </c>
+      <c r="I5">
         <v>15</v>
       </c>
-      <c r="C5">
-        <v>15</v>
-      </c>
-      <c r="D5">
-        <v>12</v>
-      </c>
-      <c r="E5">
-        <v>11</v>
-      </c>
-      <c r="F5">
-        <v>12</v>
-      </c>
-      <c r="G5">
-        <v>9</v>
-      </c>
-      <c r="H5">
-        <v>11</v>
-      </c>
-      <c r="I5">
-        <v>12</v>
-      </c>
       <c r="J5">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>9</v>
       </c>
       <c r="L5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>14</v>
+      </c>
+      <c r="C6">
+        <v>26</v>
+      </c>
+      <c r="D6">
+        <v>29</v>
+      </c>
+      <c r="E6">
+        <v>24</v>
+      </c>
+      <c r="F6">
+        <v>42</v>
+      </c>
+      <c r="G6">
+        <v>18</v>
+      </c>
+      <c r="H6">
+        <v>18</v>
+      </c>
+      <c r="I6">
+        <v>21</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
+        <v>18</v>
+      </c>
+      <c r="L6">
+        <v>18</v>
+      </c>
+      <c r="M6">
         <v>8</v>
       </c>
     </row>
@@ -20360,10 +20347,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -20423,26 +20410,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L2">
         <v>2</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -20450,124 +20452,122 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I3">
         <v>2</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L3">
+        <v>6</v>
+      </c>
+      <c r="M3">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4">
+        <v>7</v>
+      </c>
+      <c r="F4">
+        <v>7</v>
+      </c>
+      <c r="G4">
+        <v>7</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4">
+        <v>8</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C5">
+        <v>15</v>
+      </c>
+      <c r="D5">
+        <v>12</v>
+      </c>
+      <c r="E5">
         <v>11</v>
       </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-      <c r="E5">
-        <v>17</v>
-      </c>
       <c r="F5">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G5">
+        <v>9</v>
+      </c>
+      <c r="H5">
+        <v>11</v>
+      </c>
+      <c r="I5">
         <v>12</v>
       </c>
-      <c r="H5">
-        <v>12</v>
-      </c>
-      <c r="I5">
-        <v>17</v>
-      </c>
       <c r="J5">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="K5">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="L5">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="M5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>11</v>
-      </c>
-      <c r="D6">
-        <v>9</v>
-      </c>
-      <c r="E6">
-        <v>19</v>
-      </c>
-      <c r="F6">
-        <v>24</v>
-      </c>
-      <c r="G6">
-        <v>15</v>
-      </c>
-      <c r="H6">
-        <v>17</v>
-      </c>
-      <c r="I6">
-        <v>19</v>
-      </c>
-      <c r="J6">
-        <v>14</v>
-      </c>
-      <c r="K6">
-        <v>24</v>
-      </c>
-      <c r="L6">
-        <v>10</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-09-27
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
     <sheet name="Garfield Park" sheetId="3" r:id="rId3"/>
-    <sheet name="North Lawndale" sheetId="4" r:id="rId4"/>
-    <sheet name="Englewood" sheetId="5" r:id="rId5"/>
+    <sheet name="Englewood" sheetId="4" r:id="rId4"/>
+    <sheet name="North Lawndale" sheetId="5" r:id="rId5"/>
     <sheet name="Uptown" sheetId="6" r:id="rId6"/>
     <sheet name="Riverdale" sheetId="7" r:id="rId7"/>
     <sheet name="Fuller Park" sheetId="8" r:id="rId8"/>
@@ -1050,7 +1050,7 @@
         <v>467</v>
       </c>
       <c r="M6">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>896</v>
       </c>
       <c r="M7">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -4374,7 +4374,7 @@
         <v>70</v>
       </c>
       <c r="M28">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -4514,7 +4514,7 @@
         <v>44</v>
       </c>
       <c r="M32">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -6812,7 +6812,7 @@
         <v>896</v>
       </c>
       <c r="M98">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
   </sheetData>
@@ -9049,7 +9049,7 @@
         <v>31</v>
       </c>
       <c r="M6">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -9090,7 +9090,7 @@
         <v>44</v>
       </c>
       <c r="M7">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -11239,7 +11239,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -11302,41 +11302,38 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="K2">
         <v>3</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -11344,130 +11341,159 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>18</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
       <c r="H4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J4">
         <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>12</v>
-      </c>
-      <c r="C5">
-        <v>21</v>
-      </c>
-      <c r="D5">
-        <v>28</v>
-      </c>
-      <c r="E5">
-        <v>21</v>
-      </c>
-      <c r="F5">
-        <v>35</v>
-      </c>
-      <c r="G5">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I5">
-        <v>15</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>9</v>
-      </c>
-      <c r="L5">
-        <v>7</v>
-      </c>
-      <c r="M5">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="C6">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D6">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F6">
         <v>42</v>
       </c>
       <c r="G6">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="H6">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I6">
         <v>21</v>
       </c>
       <c r="J6">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K6">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="L6">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="M6">
-        <v>10</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>40</v>
+      </c>
+      <c r="C7">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>50</v>
+      </c>
+      <c r="E7">
+        <v>33</v>
+      </c>
+      <c r="F7">
+        <v>63</v>
+      </c>
+      <c r="G7">
+        <v>50</v>
+      </c>
+      <c r="H7">
+        <v>47</v>
+      </c>
+      <c r="I7">
+        <v>45</v>
+      </c>
+      <c r="J7">
+        <v>37</v>
+      </c>
+      <c r="K7">
+        <v>68</v>
+      </c>
+      <c r="L7">
+        <v>70</v>
+      </c>
+      <c r="M7">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -13543,7 +13569,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -13606,38 +13632,41 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K2">
         <v>3</v>
       </c>
       <c r="L2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -13645,159 +13674,130 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G3">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <v>6</v>
+      </c>
+      <c r="L3">
         <v>7</v>
       </c>
-      <c r="I3">
-        <v>13</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>20</v>
-      </c>
-      <c r="L3">
-        <v>20</v>
-      </c>
       <c r="M3">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
       <c r="H4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>21</v>
+      </c>
+      <c r="D5">
+        <v>28</v>
+      </c>
+      <c r="E5">
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>35</v>
+      </c>
+      <c r="G5">
+        <v>12</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>9</v>
+      </c>
+      <c r="L5">
+        <v>7</v>
+      </c>
+      <c r="M5">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="C6">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="D6">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F6">
         <v>42</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H6">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="I6">
         <v>21</v>
       </c>
       <c r="J6">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K6">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="L6">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="M6">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>40</v>
-      </c>
-      <c r="C7">
-        <v>51</v>
-      </c>
-      <c r="D7">
-        <v>50</v>
-      </c>
-      <c r="E7">
-        <v>33</v>
-      </c>
-      <c r="F7">
-        <v>63</v>
-      </c>
-      <c r="G7">
-        <v>50</v>
-      </c>
-      <c r="H7">
-        <v>47</v>
-      </c>
-      <c r="I7">
-        <v>45</v>
-      </c>
-      <c r="J7">
-        <v>37</v>
-      </c>
-      <c r="K7">
-        <v>68</v>
-      </c>
-      <c r="L7">
-        <v>70</v>
-      </c>
-      <c r="M7">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-01
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -10,20 +10,20 @@
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
     <sheet name="West Town" sheetId="3" r:id="rId3"/>
-    <sheet name="Grand Boulevard" sheetId="4" r:id="rId4"/>
-    <sheet name="Avondale" sheetId="5" r:id="rId5"/>
-    <sheet name="Mount Greenwood" sheetId="6" r:id="rId6"/>
-    <sheet name="Grand Crossing" sheetId="7" r:id="rId7"/>
-    <sheet name="Englewood" sheetId="8" r:id="rId8"/>
-    <sheet name="Washington Park" sheetId="9" r:id="rId9"/>
-    <sheet name="South Chicago" sheetId="10" r:id="rId10"/>
-    <sheet name="Humboldt Park" sheetId="11" r:id="rId11"/>
-    <sheet name="Garfield Park" sheetId="12" r:id="rId12"/>
-    <sheet name="Rush &amp; Division" sheetId="13" r:id="rId13"/>
-    <sheet name="Loop" sheetId="14" r:id="rId14"/>
-    <sheet name="United Center" sheetId="15" r:id="rId15"/>
-    <sheet name="Chatham" sheetId="16" r:id="rId16"/>
-    <sheet name="Ashburn" sheetId="17" r:id="rId17"/>
+    <sheet name="Ashburn" sheetId="4" r:id="rId4"/>
+    <sheet name="Grand Crossing" sheetId="5" r:id="rId5"/>
+    <sheet name="Englewood" sheetId="6" r:id="rId6"/>
+    <sheet name="Grand Boulevard" sheetId="7" r:id="rId7"/>
+    <sheet name="Avondale" sheetId="8" r:id="rId8"/>
+    <sheet name="Mount Greenwood" sheetId="9" r:id="rId9"/>
+    <sheet name="Washington Park" sheetId="10" r:id="rId10"/>
+    <sheet name="South Chicago" sheetId="11" r:id="rId11"/>
+    <sheet name="Humboldt Park" sheetId="12" r:id="rId12"/>
+    <sheet name="Garfield Park" sheetId="13" r:id="rId13"/>
+    <sheet name="Rush &amp; Division" sheetId="14" r:id="rId14"/>
+    <sheet name="Loop" sheetId="15" r:id="rId15"/>
+    <sheet name="United Center" sheetId="16" r:id="rId16"/>
+    <sheet name="Chatham" sheetId="17" r:id="rId17"/>
     <sheet name="South Shore" sheetId="18" r:id="rId18"/>
     <sheet name="Sheffield &amp; DePaul" sheetId="19" r:id="rId19"/>
     <sheet name="Lake View" sheetId="20" r:id="rId20"/>
@@ -889,7 +889,7 @@
         <v>137</v>
       </c>
       <c r="M2">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -930,7 +930,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>896</v>
       </c>
       <c r="M7">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
   </sheetData>
@@ -1100,6 +1100,235 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>3</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>3</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="E5">
+        <v>6</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>7</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>8</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>7</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>11</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>7</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>7</v>
+      </c>
+      <c r="I6">
+        <v>12</v>
+      </c>
+      <c r="J6">
+        <v>12</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>8</v>
+      </c>
+      <c r="M6">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1314,7 +1543,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1549,7 +1778,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1813,7 +2042,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2030,7 +2259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2315,7 +2544,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2538,7 +2767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2783,197 +3012,6 @@
       </c>
       <c r="M7">
         <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>3</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="E4">
-        <v>2</v>
-      </c>
-      <c r="F4">
-        <v>3</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>4</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>4</v>
-      </c>
-      <c r="L4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>4</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>5</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>8</v>
-      </c>
-      <c r="J5">
-        <v>3</v>
-      </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="L5">
-        <v>9</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4359,7 +4397,7 @@
         <v>70</v>
       </c>
       <c r="M28">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -4612,7 +4650,7 @@
         <v>63</v>
       </c>
       <c r="M36">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -6797,7 +6835,7 @@
         <v>896</v>
       </c>
       <c r="M98">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
   </sheetData>
@@ -11607,7 +11645,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -11671,150 +11709,124 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="I2">
         <v>2</v>
       </c>
       <c r="L2">
         <v>2</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
       <c r="I3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
         <v>1</v>
       </c>
       <c r="L3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
+      </c>
+      <c r="G4">
+        <v>3</v>
       </c>
       <c r="H4">
         <v>1</v>
+      </c>
+      <c r="I4">
+        <v>4</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="I5">
         <v>8</v>
       </c>
-      <c r="E5">
-        <v>5</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>6</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
       <c r="J5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
         <v>9</v>
       </c>
-      <c r="C6">
-        <v>13</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>6</v>
-      </c>
-      <c r="F6">
-        <v>8</v>
-      </c>
-      <c r="G6">
-        <v>7</v>
-      </c>
-      <c r="H6">
-        <v>5</v>
-      </c>
-      <c r="I6">
-        <v>6</v>
-      </c>
-      <c r="J6">
-        <v>8</v>
-      </c>
-      <c r="K6">
-        <v>9</v>
-      </c>
-      <c r="L6">
-        <v>12</v>
-      </c>
-      <c r="M6">
-        <v>5</v>
+      <c r="M5">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -13745,7 +13757,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -13809,144 +13821,200 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
       <c r="E3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>17</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="K4">
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="M4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-      <c r="G5">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>5</v>
-      </c>
       <c r="I5">
-        <v>3</v>
-      </c>
-      <c r="J5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L5">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="J6">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7">
+        <v>42</v>
+      </c>
+      <c r="D7">
+        <v>36</v>
+      </c>
+      <c r="E7">
+        <v>38</v>
+      </c>
+      <c r="F7">
+        <v>53</v>
+      </c>
+      <c r="G7">
+        <v>28</v>
+      </c>
+      <c r="H7">
+        <v>39</v>
+      </c>
+      <c r="I7">
+        <v>39</v>
+      </c>
+      <c r="J7">
+        <v>47</v>
+      </c>
+      <c r="K7">
+        <v>74</v>
+      </c>
+      <c r="L7">
+        <v>63</v>
+      </c>
+      <c r="M7">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -15546,60 +15614,261 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
         <v>2016</v>
       </c>
-      <c r="C1" s="1">
+      <c r="D1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="D1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="K1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="M1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
       <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
+      </c>
+      <c r="H2">
+        <v>11</v>
+      </c>
+      <c r="I2">
+        <v>10</v>
+      </c>
+      <c r="J2">
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
+      </c>
+      <c r="L2">
+        <v>6</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>18</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>12</v>
+      </c>
+      <c r="G3">
+        <v>11</v>
+      </c>
+      <c r="H3">
+        <v>7</v>
+      </c>
+      <c r="I3">
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
+      </c>
+      <c r="K3">
+        <v>20</v>
+      </c>
+      <c r="L3">
+        <v>20</v>
+      </c>
+      <c r="M3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
       <c r="D4">
         <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>45</v>
+      </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <v>22</v>
+      </c>
+      <c r="F6">
+        <v>42</v>
+      </c>
+      <c r="G6">
+        <v>32</v>
+      </c>
+      <c r="H6">
+        <v>26</v>
+      </c>
+      <c r="I6">
+        <v>21</v>
+      </c>
+      <c r="J6">
+        <v>15</v>
+      </c>
+      <c r="K6">
+        <v>44</v>
+      </c>
+      <c r="L6">
+        <v>43</v>
+      </c>
+      <c r="M6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>40</v>
+      </c>
+      <c r="C7">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>50</v>
+      </c>
+      <c r="E7">
+        <v>33</v>
+      </c>
+      <c r="F7">
+        <v>63</v>
+      </c>
+      <c r="G7">
+        <v>50</v>
+      </c>
+      <c r="H7">
+        <v>47</v>
+      </c>
+      <c r="I7">
+        <v>45</v>
+      </c>
+      <c r="J7">
+        <v>37</v>
+      </c>
+      <c r="K7">
+        <v>68</v>
+      </c>
+      <c r="L7">
+        <v>70</v>
+      </c>
+      <c r="M7">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -17332,10 +17601,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
@@ -17395,41 +17664,29 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H2">
-        <v>6</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -17437,159 +17694,121 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>8</v>
-      </c>
-      <c r="E3">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>9</v>
-      </c>
-      <c r="H3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="L3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>2</v>
-      </c>
-      <c r="M4">
+        <v>4</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>6</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="C6">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="F6">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="G6">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="H6">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="J6">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="K6">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="L6">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="M6">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>32</v>
-      </c>
-      <c r="C7">
-        <v>42</v>
-      </c>
-      <c r="D7">
-        <v>36</v>
-      </c>
-      <c r="E7">
-        <v>38</v>
-      </c>
-      <c r="F7">
-        <v>53</v>
-      </c>
-      <c r="G7">
-        <v>28</v>
-      </c>
-      <c r="H7">
-        <v>39</v>
-      </c>
-      <c r="I7">
-        <v>39</v>
-      </c>
-      <c r="J7">
-        <v>47</v>
-      </c>
-      <c r="K7">
-        <v>74</v>
-      </c>
-      <c r="L7">
-        <v>63</v>
-      </c>
-      <c r="M7">
-        <v>27</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -18960,7 +19179,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -19023,79 +19242,55 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>18</v>
-      </c>
       <c r="E3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>11</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="L3">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -19105,116 +19300,87 @@
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
       <c r="K4">
         <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
         <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="J5">
+        <v>6</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="J6">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="K6">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="L6">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>40</v>
-      </c>
-      <c r="C7">
-        <v>51</v>
-      </c>
-      <c r="D7">
-        <v>50</v>
-      </c>
-      <c r="E7">
-        <v>33</v>
-      </c>
-      <c r="F7">
-        <v>63</v>
-      </c>
-      <c r="G7">
-        <v>50</v>
-      </c>
-      <c r="H7">
-        <v>47</v>
-      </c>
-      <c r="I7">
-        <v>45</v>
-      </c>
-      <c r="J7">
-        <v>37</v>
-      </c>
-      <c r="K7">
-        <v>68</v>
-      </c>
-      <c r="L7">
-        <v>70</v>
-      </c>
-      <c r="M7">
-        <v>28</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -20328,226 +20494,60 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" customWidth="1"/>
     <col min="3" max="3" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="C1" s="1">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
       <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>3</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>1</v>
-      </c>
-      <c r="M2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
-      </c>
-      <c r="I3">
-        <v>3</v>
-      </c>
-      <c r="J3">
-        <v>4</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>5</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>7</v>
-      </c>
-      <c r="D5">
-        <v>7</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>7</v>
-      </c>
-      <c r="H5">
-        <v>4</v>
-      </c>
-      <c r="I5">
-        <v>8</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>7</v>
-      </c>
-      <c r="C6">
-        <v>10</v>
-      </c>
-      <c r="D6">
-        <v>11</v>
-      </c>
-      <c r="E6">
-        <v>10</v>
-      </c>
-      <c r="F6">
-        <v>7</v>
-      </c>
-      <c r="G6">
-        <v>10</v>
-      </c>
-      <c r="H6">
-        <v>7</v>
-      </c>
-      <c r="I6">
-        <v>12</v>
-      </c>
-      <c r="J6">
-        <v>12</v>
-      </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
-        <v>8</v>
-      </c>
-      <c r="M6">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add data for 2026-10-20
</commit_message>
<xml_diff>
--- a/output/cta-violent-crime-full-year.xlsx
+++ b/output/cta-violent-crime-full-year.xlsx
@@ -9,16 +9,16 @@
   <sheets>
     <sheet name="Citywide Totals" sheetId="1" r:id="rId1"/>
     <sheet name="By Neighborhood" sheetId="2" r:id="rId2"/>
-    <sheet name="Douglas" sheetId="3" r:id="rId3"/>
-    <sheet name="Austin" sheetId="4" r:id="rId4"/>
-    <sheet name="Garfield Park" sheetId="5" r:id="rId5"/>
-    <sheet name="Little Italy, UIC" sheetId="6" r:id="rId6"/>
-    <sheet name="West Loop" sheetId="7" r:id="rId7"/>
-    <sheet name="Loop" sheetId="8" r:id="rId8"/>
-    <sheet name="Wicker Park" sheetId="9" r:id="rId9"/>
-    <sheet name="Roseland" sheetId="10" r:id="rId10"/>
-    <sheet name="West Town" sheetId="11" r:id="rId11"/>
-    <sheet name="Englewood" sheetId="12" r:id="rId12"/>
+    <sheet name="Englewood" sheetId="3" r:id="rId3"/>
+    <sheet name="West Loop" sheetId="4" r:id="rId4"/>
+    <sheet name="Roseland" sheetId="5" r:id="rId5"/>
+    <sheet name="Douglas" sheetId="6" r:id="rId6"/>
+    <sheet name="Austin" sheetId="7" r:id="rId7"/>
+    <sheet name="Garfield Park" sheetId="8" r:id="rId8"/>
+    <sheet name="Little Italy, UIC" sheetId="9" r:id="rId9"/>
+    <sheet name="Loop" sheetId="10" r:id="rId10"/>
+    <sheet name="Wicker Park" sheetId="11" r:id="rId11"/>
+    <sheet name="West Town" sheetId="12" r:id="rId12"/>
     <sheet name="Grand Crossing" sheetId="13" r:id="rId13"/>
     <sheet name="Auburn Gresham" sheetId="14" r:id="rId14"/>
     <sheet name="Woodlawn" sheetId="15" r:id="rId15"/>
@@ -930,7 +930,7 @@
         <v>262</v>
       </c>
       <c r="M3">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1050,7 +1050,7 @@
         <v>467</v>
       </c>
       <c r="M6">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1091,7 +1091,7 @@
         <v>896</v>
       </c>
       <c r="M7">
-        <v>508</v>
+        <v>511</v>
       </c>
     </row>
   </sheetData>
@@ -1165,37 +1165,37 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I2">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="K2">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="M2">
         <v>2</v>
@@ -1206,40 +1206,40 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="F3">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G3">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="I3">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J3">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="K3">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="L3">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="M3">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1247,32 +1247,53 @@
         <v>3</v>
       </c>
       <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
       </c>
       <c r="I4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
+      <c r="M5">
         <v>1</v>
       </c>
     </row>
@@ -1281,40 +1302,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C6">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="D6">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E6">
-        <v>14</v>
+        <v>67</v>
       </c>
       <c r="F6">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="G6">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="H6">
-        <v>19</v>
+        <v>80</v>
       </c>
       <c r="I6">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="J6">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="K6">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="L6">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="M6">
-        <v>7</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1322,40 +1343,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="C7">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="D7">
-        <v>16</v>
+        <v>79</v>
       </c>
       <c r="E7">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="F7">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="G7">
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="H7">
-        <v>31</v>
+        <v>120</v>
       </c>
       <c r="I7">
+        <v>130</v>
+      </c>
+      <c r="J7">
+        <v>131</v>
+      </c>
+      <c r="K7">
+        <v>91</v>
+      </c>
+      <c r="L7">
+        <v>100</v>
+      </c>
+      <c r="M7">
         <v>47</v>
-      </c>
-      <c r="J7">
-        <v>35</v>
-      </c>
-      <c r="K7">
-        <v>31</v>
-      </c>
-      <c r="L7">
-        <v>37</v>
-      </c>
-      <c r="M7">
-        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1364,6 +1385,186 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="4.7109375" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" customWidth="1"/>
+    <col min="8" max="8" width="4.7109375" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" customWidth="1"/>
+    <col min="10" max="10" width="4.7109375" customWidth="1"/>
+    <col min="11" max="11" width="4.7109375" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2016</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2017</v>
+      </c>
+      <c r="D1" s="1">
+        <v>2018</v>
+      </c>
+      <c r="E1" s="1">
+        <v>2019</v>
+      </c>
+      <c r="F1" s="1">
+        <v>2020</v>
+      </c>
+      <c r="G1" s="1">
+        <v>2021</v>
+      </c>
+      <c r="H1" s="1">
+        <v>2022</v>
+      </c>
+      <c r="I1" s="1">
+        <v>2023</v>
+      </c>
+      <c r="J1" s="1">
+        <v>2024</v>
+      </c>
+      <c r="K1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="L1" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+      <c r="D6">
+        <v>6</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <v>6</v>
+      </c>
+      <c r="I6">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1585,270 +1786,6 @@
       </c>
       <c r="M6">
         <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" customWidth="1"/>
-    <col min="4" max="4" width="4.7109375" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" customWidth="1"/>
-    <col min="6" max="6" width="4.7109375" customWidth="1"/>
-    <col min="7" max="7" width="4.7109375" customWidth="1"/>
-    <col min="8" max="8" width="4.7109375" customWidth="1"/>
-    <col min="9" max="9" width="4.7109375" customWidth="1"/>
-    <col min="10" max="10" width="4.7109375" customWidth="1"/>
-    <col min="11" max="11" width="4.7109375" customWidth="1"/>
-    <col min="12" max="12" width="4.7109375" customWidth="1"/>
-    <col min="13" max="13" width="4.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1">
-        <v>2015</v>
-      </c>
-      <c r="C1" s="1">
-        <v>2016</v>
-      </c>
-      <c r="D1" s="1">
-        <v>2017</v>
-      </c>
-      <c r="E1" s="1">
-        <v>2018</v>
-      </c>
-      <c r="F1" s="1">
-        <v>2019</v>
-      </c>
-      <c r="G1" s="1">
-        <v>2020</v>
-      </c>
-      <c r="H1" s="1">
-        <v>2021</v>
-      </c>
-      <c r="I1" s="1">
-        <v>2022</v>
-      </c>
-      <c r="J1" s="1">
-        <v>2023</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2024</v>
-      </c>
-      <c r="L1" s="1">
-        <v>2025</v>
-      </c>
-      <c r="M1" s="1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>6</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
-      </c>
-      <c r="G2">
-        <v>7</v>
-      </c>
-      <c r="H2">
-        <v>11</v>
-      </c>
-      <c r="I2">
-        <v>10</v>
-      </c>
-      <c r="J2">
-        <v>9</v>
-      </c>
-      <c r="K2">
-        <v>3</v>
-      </c>
-      <c r="L2">
-        <v>6</v>
-      </c>
-      <c r="M2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>18</v>
-      </c>
-      <c r="E3">
-        <v>10</v>
-      </c>
-      <c r="F3">
-        <v>12</v>
-      </c>
-      <c r="G3">
-        <v>11</v>
-      </c>
-      <c r="H3">
-        <v>7</v>
-      </c>
-      <c r="I3">
-        <v>13</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>20</v>
-      </c>
-      <c r="L3">
-        <v>20</v>
-      </c>
-      <c r="M3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
-      <c r="A5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
-      <c r="A6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>34</v>
-      </c>
-      <c r="C6">
-        <v>45</v>
-      </c>
-      <c r="D6">
-        <v>25</v>
-      </c>
-      <c r="E6">
-        <v>22</v>
-      </c>
-      <c r="F6">
-        <v>42</v>
-      </c>
-      <c r="G6">
-        <v>32</v>
-      </c>
-      <c r="H6">
-        <v>26</v>
-      </c>
-      <c r="I6">
-        <v>21</v>
-      </c>
-      <c r="J6">
-        <v>15</v>
-      </c>
-      <c r="K6">
-        <v>44</v>
-      </c>
-      <c r="L6">
-        <v>43</v>
-      </c>
-      <c r="M6">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>40</v>
-      </c>
-      <c r="C7">
-        <v>51</v>
-      </c>
-      <c r="D7">
-        <v>50</v>
-      </c>
-      <c r="E7">
-        <v>33</v>
-      </c>
-      <c r="F7">
-        <v>63</v>
-      </c>
-      <c r="G7">
-        <v>50</v>
-      </c>
-      <c r="H7">
-        <v>47</v>
-      </c>
-      <c r="I7">
-        <v>45</v>
-      </c>
-      <c r="J7">
-        <v>37</v>
-      </c>
-      <c r="K7">
-        <v>68</v>
-      </c>
-      <c r="L7">
-        <v>70</v>
-      </c>
-      <c r="M7">
-        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -4421,7 +4358,7 @@
         <v>70</v>
       </c>
       <c r="M28">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -5284,7 +5221,7 @@
         <v>100</v>
       </c>
       <c r="M53">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -5519,7 +5456,7 @@
         <v>9</v>
       </c>
       <c r="M61">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:13">
@@ -6091,7 +6028,7 @@
         <v>37</v>
       </c>
       <c r="M77">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="78" spans="1:13">
@@ -6599,7 +6536,7 @@
         <v>14</v>
       </c>
       <c r="M91">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="92" spans="1:13">
@@ -6862,7 +6799,7 @@
         <v>896</v>
       </c>
       <c r="M98">
-        <v>508</v>
+        <v>511</v>
       </c>
     </row>
   </sheetData>
@@ -9019,25 +8956,37 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>7</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -9045,43 +8994,76 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>13</v>
+      </c>
+      <c r="J3">
+        <v>12</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>20</v>
+      </c>
+      <c r="L3">
+        <v>20</v>
       </c>
       <c r="M3">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
       <c r="J4">
         <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K5">
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
@@ -9090,37 +9072,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="J6">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="L6">
-        <v>6</v>
+        <v>43</v>
+      </c>
+      <c r="M6">
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -9128,40 +9113,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="F7">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="I7">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="J7">
-        <v>4</v>
+        <v>37</v>
       </c>
       <c r="K7">
-        <v>7</v>
+        <v>68</v>
       </c>
       <c r="L7">
-        <v>7</v>
+        <v>70</v>
       </c>
       <c r="M7">
-        <v>4</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -11284,40 +11269,31 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -11325,70 +11301,58 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K3">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
+      <c r="F4">
         <v>1</v>
       </c>
       <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="M4">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="K5">
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
@@ -11397,40 +11361,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="G6">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="I6">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="J6">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="L6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -11438,40 +11402,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C7">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D7">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="E7">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="F7">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="G7">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="H7">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="I7">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="J7">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="K7">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="L7">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="M7">
-        <v>40</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -13338,40 +13302,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>6</v>
+      </c>
+      <c r="I2">
         <v>7</v>
       </c>
-      <c r="E2">
-        <v>8</v>
-      </c>
-      <c r="F2">
-        <v>5</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>5</v>
-      </c>
       <c r="J2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -13379,25 +13343,25 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G3">
         <v>6</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I3">
         <v>9</v>
@@ -13406,36 +13370,36 @@
         <v>14</v>
       </c>
       <c r="K3">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M3">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="H4">
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="G4">
         <v>1</v>
       </c>
       <c r="I4">
         <v>2</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -13445,7 +13409,7 @@
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I5">
+      <c r="D5">
         <v>1</v>
       </c>
     </row>
@@ -13454,40 +13418,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C6">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="D6">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E6">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="F6">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="G6">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="H6">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="I6">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="J6">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="K6">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="L6">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="M6">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -13495,40 +13459,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C7">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="D7">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="E7">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="G7">
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <v>31</v>
+      </c>
+      <c r="I7">
         <v>47</v>
       </c>
-      <c r="H7">
-        <v>50</v>
-      </c>
-      <c r="I7">
-        <v>49</v>
-      </c>
       <c r="J7">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="K7">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="L7">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="M7">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -15129,7 +15093,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -15193,31 +15157,25 @@
         <v>1</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J2">
-        <v>1</v>
-      </c>
-      <c r="K2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -15225,139 +15183,123 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
       <c r="F3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>4</v>
-      </c>
-      <c r="J3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
-      </c>
-      <c r="K4">
-        <v>3</v>
-      </c>
-      <c r="L4">
-        <v>1</v>
-      </c>
-      <c r="M4">
+      <c r="J4">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>7</v>
-      </c>
-      <c r="D5">
-        <v>11</v>
-      </c>
-      <c r="E5">
-        <v>21</v>
-      </c>
-      <c r="F5">
-        <v>25</v>
-      </c>
-      <c r="G5">
-        <v>15</v>
-      </c>
-      <c r="H5">
-        <v>10</v>
-      </c>
-      <c r="I5">
-        <v>9</v>
-      </c>
-      <c r="J5">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>18</v>
-      </c>
-      <c r="L5">
-        <v>11</v>
-      </c>
-      <c r="M5">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F6">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="G6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="L6">
-        <v>22</v>
-      </c>
-      <c r="M6">
-        <v>15</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>7</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>8</v>
+      </c>
+      <c r="I7">
+        <v>7</v>
+      </c>
+      <c r="J7">
+        <v>4</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -17180,31 +17122,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -17212,55 +17163,70 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>14</v>
+      </c>
+      <c r="M3">
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F4">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
         <v>1</v>
       </c>
       <c r="J4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I5">
+      <c r="K5">
         <v>1</v>
       </c>
     </row>
@@ -17269,40 +17235,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="E6">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="G6">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="H6">
-        <v>9</v>
+        <v>50</v>
       </c>
       <c r="I6">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="M6">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -17310,40 +17276,40 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="E7">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="F7">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="G7">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="H7">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="I7">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="J7">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="K7">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="L7">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -19013,40 +18979,40 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G2">
         <v>4</v>
       </c>
       <c r="H2">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="J2">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="M2">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -19054,94 +19020,73 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C3">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E3">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>6</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>9</v>
+      </c>
+      <c r="J3">
         <v>14</v>
       </c>
-      <c r="G3">
-        <v>26</v>
-      </c>
-      <c r="H3">
-        <v>23</v>
-      </c>
-      <c r="I3">
-        <v>32</v>
-      </c>
-      <c r="J3">
-        <v>40</v>
-      </c>
       <c r="K3">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="L3">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="M3">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4">
+      <c r="B4">
         <v>2</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>4</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="L5">
-        <v>2</v>
-      </c>
-      <c r="M5">
+      <c r="I5">
         <v>1</v>
       </c>
     </row>
@@ -19150,40 +19095,40 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="D6">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="E6">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F6">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="G6">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="H6">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="I6">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="J6">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="K6">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="L6">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="M6">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -19191,40 +19136,40 @@
         <v>6</v>
       </c>
       <c r="B7">
+        <v>19</v>
+      </c>
+      <c r="C7">
+        <v>40</v>
+      </c>
+      <c r="D7">
+        <v>51</v>
+      </c>
+      <c r="E7">
+        <v>69</v>
+      </c>
+      <c r="F7">
+        <v>65</v>
+      </c>
+      <c r="G7">
+        <v>47</v>
+      </c>
+      <c r="H7">
+        <v>50</v>
+      </c>
+      <c r="I7">
         <v>49</v>
       </c>
-      <c r="C7">
-        <v>62</v>
-      </c>
-      <c r="D7">
-        <v>79</v>
-      </c>
-      <c r="E7">
-        <v>92</v>
-      </c>
-      <c r="F7">
-        <v>92</v>
-      </c>
-      <c r="G7">
-        <v>88</v>
-      </c>
-      <c r="H7">
-        <v>120</v>
-      </c>
-      <c r="I7">
-        <v>130</v>
-      </c>
       <c r="J7">
-        <v>131</v>
+        <v>51</v>
       </c>
       <c r="K7">
-        <v>91</v>
+        <v>48</v>
       </c>
       <c r="L7">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="M7">
-        <v>46</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -20421,7 +20366,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
@@ -20436,162 +20381,220 @@
     <col min="10" max="10" width="4.7109375" customWidth="1"/>
     <col min="11" max="11" width="4.7109375" customWidth="1"/>
     <col min="12" max="12" width="4.7109375" customWidth="1"/>
+    <col min="13" max="13" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
+        <v>2015</v>
+      </c>
+      <c r="C1" s="1">
         <v>2016</v>
       </c>
-      <c r="C1" s="1">
+      <c r="D1" s="1">
         <v>2017</v>
       </c>
-      <c r="D1" s="1">
+      <c r="E1" s="1">
         <v>2018</v>
       </c>
-      <c r="E1" s="1">
+      <c r="F1" s="1">
         <v>2019</v>
       </c>
-      <c r="F1" s="1">
+      <c r="G1" s="1">
         <v>2020</v>
       </c>
-      <c r="G1" s="1">
+      <c r="H1" s="1">
         <v>2021</v>
       </c>
-      <c r="H1" s="1">
+      <c r="I1" s="1">
         <v>2022</v>
       </c>
-      <c r="I1" s="1">
+      <c r="J1" s="1">
         <v>2023</v>
       </c>
-      <c r="J1" s="1">
+      <c r="K1" s="1">
         <v>2024</v>
       </c>
-      <c r="K1" s="1">
+      <c r="L1" s="1">
         <v>2025</v>
       </c>
-      <c r="L1" s="1">
+      <c r="M1" s="1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
       </c>
       <c r="L2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>4</v>
+      </c>
+      <c r="M2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
       <c r="D3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
       </c>
       <c r="L3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
+        <v>6</v>
+      </c>
+      <c r="M3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>3</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>21</v>
+      </c>
+      <c r="F5">
+        <v>25</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="H5">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="J5">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+        <v>18</v>
+      </c>
+      <c r="L5">
+        <v>11</v>
+      </c>
+      <c r="M5">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H6">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I6">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="K6">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>22</v>
+      </c>
+      <c r="M6">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>